<commit_message>
fix(batch): correct cohort graduation metrics, topper multi-sem deduplication, and trajectory classification
</commit_message>
<xml_diff>
--- a/departments_data/excel/Artificial_Intelligence_and_Data_Science/21-22/Sem_1.xlsx
+++ b/departments_data/excel/Artificial_Intelligence_and_Data_Science/21-22/Sem_1.xlsx
@@ -434,7 +434,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -493,13 +493,21 @@
           <t>9041687</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NILESH RAMAVTAR YADAV</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>2021016402170572</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F2" t="n">
         <v>9.56</v>
       </c>
@@ -519,13 +527,21 @@
           <t>9041688</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DHANDE NITESH RAMESH</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>2021016402156235</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F3" t="n">
         <v>9.58</v>
       </c>
@@ -545,13 +561,21 @@
           <t>9041689</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ADULKAR VEDANT SANJAY</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>2021016402160442</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F4" t="n">
         <v>9.359999999999999</v>
       </c>
@@ -571,13 +595,21 @@
           <t>9041690</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>AJANI ALI MEHDI AZHAR HUSAIN</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>2021016402156394</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F5" t="n">
         <v>9.33</v>
       </c>
@@ -597,13 +629,21 @@
           <t>9041691</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PRIYANKA VIVEK ANGANE</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>2021016402160152</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F6" t="n">
         <v>8.970000000000001</v>
       </c>
@@ -623,13 +663,21 @@
           <t>9041692</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>JATIN BANDEKAR</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>2021016402164165</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F7" t="n">
         <v>9.67</v>
       </c>
@@ -649,13 +697,21 @@
           <t>9041693</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>BANSODE AADITYA RHIDAYNATH</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>2021016402156034</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F8" t="n">
         <v>9.279999999999999</v>
       </c>
@@ -675,13 +731,21 @@
           <t>9041694</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BANSODE SAMRUDDHI PARSHURAM</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>2021016402157111</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F9" t="n">
         <v>9.58</v>
       </c>
@@ -701,13 +765,21 @@
           <t>9041695</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BENKE PARTH NILESH</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>2021016402150834</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F10" t="n">
         <v>9.109999999999999</v>
       </c>
@@ -727,13 +799,21 @@
           <t>9041696</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>KU SANIKA</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>2021016402164993</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F11" t="n">
         <v>9.33</v>
       </c>
@@ -753,13 +833,21 @@
           <t>9041697</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>BHAMRE SHANKHIN DEEPAK</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>2021016402165315</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F12" t="n">
         <v>8.58</v>
       </c>
@@ -779,13 +867,21 @@
           <t>9041698</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CHAUDHARI PRAJAKTA</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>2021016402156073</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F13" t="n">
         <v>8.970000000000001</v>
       </c>
@@ -805,13 +901,21 @@
           <t>9041699</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MANASI SURESH DALAVI</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>2021016402156765</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F14" t="n">
         <v>9.56</v>
       </c>
@@ -831,13 +935,21 @@
           <t>9041700</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DALVI VEDANT SANDESH</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>2021016402150803</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F15" t="n">
         <v>9.44</v>
       </c>
@@ -857,13 +969,21 @@
           <t>9041701</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>DANDGE ATHARVA ANIL</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>2021016402148835</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F16" t="n">
         <v>9.109999999999999</v>
       </c>
@@ -883,13 +1003,21 @@
           <t>9041702</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CHAITANYA RAJENDRA DEOKAR</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>2021016402160113</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F17" t="n">
         <v>8.640000000000001</v>
       </c>
@@ -909,13 +1037,21 @@
           <t>9041703</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DIDWAGH AKASH BALU</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>2021016402158234</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F18" t="n">
         <v>9.720000000000001</v>
       </c>
@@ -935,13 +1071,21 @@
           <t>9041704</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>NIHAL DUBE</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>2021016402158892</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F19" t="n">
         <v>9.33</v>
       </c>
@@ -961,13 +1105,21 @@
           <t>9041705</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FALE PRANAV GAJANAN</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>2021016402157092</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F20" t="n">
         <v>9.31</v>
       </c>
@@ -987,13 +1139,21 @@
           <t>9041706</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>GAYATRI CHANDRASEN GIDE</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>2021016402156711</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F21" t="n">
         <v>8.83</v>
       </c>
@@ -1013,13 +1173,21 @@
           <t>9041707</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>GUPTA ABHAYCHANDRA</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>2021016402156421</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F22" t="n">
         <v>9.779999999999999</v>
       </c>
@@ -1039,20 +1207,24 @@
           <t>9041708</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SURYANSH JAYPRAKASH GUPTA</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>2021016402166454</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>8.50</t>
-        </is>
-      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H23" t="n">
         <v>241</v>
@@ -1067,13 +1239,21 @@
           <t>9041709</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>HAYYAN ASLAM HAJWANI</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>2021016402164142</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F24" t="n">
         <v>9.75</v>
       </c>
@@ -1093,20 +1273,24 @@
           <t>9041710</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>VINEET DINKAR HANKARE</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>2021016402150792</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>8.17</t>
-        </is>
-      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H25" t="n">
         <v>232</v>
@@ -1121,13 +1305,21 @@
           <t>9041711</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>HINUKALE VIVEK SUNIL</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>2021016402164641</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F26" t="n">
         <v>9.359999999999999</v>
       </c>
@@ -1147,13 +1339,21 @@
           <t>9041712</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>JADHAV AJINKYA SURESH</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>2021016401713915</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F27" t="n">
         <v>8.67</v>
       </c>
@@ -1173,13 +1373,21 @@
           <t>9041713</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>JADHAV ROHAN PRAVIN</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>2021016402151942</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F28" t="n">
         <v>8.06</v>
       </c>
@@ -1199,13 +1407,21 @@
           <t>9041714</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>JAGDALE ADITYA SUNIL</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>2021016402161921</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F29" t="n">
         <v>8.800000000000001</v>
       </c>
@@ -1225,13 +1441,21 @@
           <t>9041715</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>RAJ VIKAS JAISWAR</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>2021016402148827</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F30" t="n">
         <v>9.390000000000001</v>
       </c>
@@ -1251,13 +1475,21 @@
           <t>9041716</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>JATTI SOMESH RAMDAS</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>2021016402164656</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F31" t="n">
         <v>9.800000000000001</v>
       </c>
@@ -1277,13 +1509,21 @@
           <t>9041717</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>VEDANT NIHAL KADAM</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>2021016402148522</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F32" t="n">
         <v>8.970000000000001</v>
       </c>
@@ -1303,20 +1543,24 @@
           <t>9041718</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>KASKAR KHUSHI KALPESH</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>2021016400340985</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>8.22</t>
-        </is>
-      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H33" t="n">
         <v>233</v>
@@ -1331,13 +1575,21 @@
           <t>9041719</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>KHAN SUFIYAN JAHIRUDDIN</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>2021016402156026</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F34" t="n">
         <v>9.609999999999999</v>
       </c>
@@ -1357,13 +1609,21 @@
           <t>9041720</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>KOCHAREKAR ATHARVA TUKARAM</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>2021016402161317</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F35" t="n">
         <v>9.359999999999999</v>
       </c>
@@ -1383,13 +1643,21 @@
           <t>9041721</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>SHLOK NANDKUMAR KUNDALE</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>2021016402154116</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F36" t="n">
         <v>9.56</v>
       </c>
@@ -1409,18 +1677,26 @@
           <t>9041722</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>MAGAR SAIRAJ RAKESH</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>2021016402166446</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="F37" t="n">
         <v>9.220000000000001</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H37" t="n">
         <v>554</v>
@@ -1435,13 +1711,21 @@
           <t>9041723</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>KHAN MAHMOODURRAHMAN</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>2021016402164126</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F38" t="n">
         <v>9.08</v>
       </c>
@@ -1461,18 +1745,26 @@
           <t>9041724</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>MASAL SANJAY PRITAM</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr">
         <is>
           <t>2021016402160933</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="F39" t="n">
         <v>8.92</v>
       </c>
       <c r="G39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H39" t="n">
         <v>525</v>
@@ -1487,13 +1779,21 @@
           <t>9041725</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>MAURYA VISHAL BAIJNATH</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr">
         <is>
           <t>2021016402158265</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F40" t="n">
         <v>9.359999999999999</v>
       </c>
@@ -1513,13 +1813,21 @@
           <t>9041726</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>MESHRAM RUPAL MUNESHWAR</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr">
         <is>
           <t>2021016402156057</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F41" t="n">
         <v>8.81</v>
       </c>
@@ -1539,18 +1847,26 @@
           <t>9041727</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>MHATRE HARSHIT MANOHAR</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr">
         <is>
           <t>2021016402164985</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
       <c r="F42" t="n">
         <v>9.75</v>
       </c>
       <c r="G42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H42" t="n">
         <v>571</v>
@@ -1565,13 +1881,21 @@
           <t>9041728</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr"/>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SRUSHTI BALARAM MHATRE</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr">
         <is>
           <t>2021016402161333</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F43" t="n">
         <v>9.890000000000001</v>
       </c>
@@ -1591,13 +1915,21 @@
           <t>9041729</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>YASH KALIDAS MOKAL</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr">
         <is>
           <t>2021016402158114</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F44" t="n">
         <v>9.92</v>
       </c>
@@ -1617,20 +1949,24 @@
           <t>9041730</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>MORE PARTH SATISH</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr">
         <is>
           <t>2021016402161936</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>7.92</t>
-        </is>
-      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H45" t="n">
         <v>472</v>
@@ -1645,13 +1981,21 @@
           <t>9041731</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr"/>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>DEVIKA PARAG PATIL</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr">
         <is>
           <t>2021016402156452</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F46" t="n">
         <v>9.779999999999999</v>
       </c>
@@ -1671,13 +2015,21 @@
           <t>9041732</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PATIL NIRAJ SANTOSH</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr">
         <is>
           <t>2021016402164157</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F47" t="n">
         <v>9.640000000000001</v>
       </c>
@@ -1697,13 +2049,21 @@
           <t>9041733</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PATIL SUJAL MAHESH</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr">
         <is>
           <t>2021016402160682</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F48" t="n">
         <v>9.06</v>
       </c>
@@ -1723,13 +2083,21 @@
           <t>9041734</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PAWAR DHANASHREE VIJAY</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr">
         <is>
           <t>2021016402157006</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F49" t="n">
         <v>9.56</v>
       </c>
@@ -1749,20 +2117,24 @@
           <t>9041735</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>RAHI AJAY CHANDRAKANT</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr">
         <is>
           <t>2021016402150811</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>2.08</t>
-        </is>
-      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H50" t="n">
         <v>235</v>
@@ -1777,13 +2149,21 @@
           <t>9041736</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>RANALKAR MANAS SANJAY</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr">
         <is>
           <t>2021016402155093</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F51" t="n">
         <v>9.140000000000001</v>
       </c>
@@ -1803,13 +2183,21 @@
           <t>9041737</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr"/>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>DEEP RANE</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
           <t>2021016402161623</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F52" t="n">
         <v>9.42</v>
       </c>
@@ -1829,13 +2217,21 @@
           <t>9041738</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr"/>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ARYA RAUT</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
           <t>2021016402160457</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F53" t="n">
         <v>10</v>
       </c>
@@ -1855,13 +2251,21 @@
           <t>9041739</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>SIDDHESH SUNIL SANAP</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
           <t>2021016402148843</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F54" t="n">
         <v>9.359999999999999</v>
       </c>
@@ -1881,13 +2285,21 @@
           <t>9041740</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr"/>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>SAWANT SUMEDH SUBHASH</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr">
         <is>
           <t>2021016402155077</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F55" t="n">
         <v>9.06</v>
       </c>
@@ -1907,13 +2319,21 @@
           <t>9041741</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>SAYED MOHAMMED HAZIQUE</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr">
         <is>
           <t>2021016402165296</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F56" t="n">
         <v>9.640000000000001</v>
       </c>
@@ -1933,13 +2353,21 @@
           <t>9041742</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SINGH AMAN JAY</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr">
         <is>
           <t>2021016402156011</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F57" t="n">
         <v>9.31</v>
       </c>
@@ -1959,13 +2387,21 @@
           <t>9041743</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr"/>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>SINGH ARPIT AJIT</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr">
         <is>
           <t>2021016402156475</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F58" t="n">
         <v>10</v>
       </c>
@@ -1985,13 +2421,21 @@
           <t>9041744</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SINGH VASUDHA CHANDRABHAN</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
           <t>2021016402152887</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F59" t="n">
         <v>9.69</v>
       </c>
@@ -2011,13 +2455,21 @@
           <t>9041745</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TAMBE TANUJ SUNIL</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
           <t>2021016402155104</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F60" t="n">
         <v>8.81</v>
       </c>
@@ -2037,13 +2489,21 @@
           <t>9041746</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>TANPURE VEDANT RAJARAM</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr">
         <is>
           <t>2021016402158497</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F61" t="n">
         <v>9.359999999999999</v>
       </c>
@@ -2063,13 +2523,21 @@
           <t>9041747</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>THAKUR DIKSHA JITENDRA</t>
+        </is>
+      </c>
       <c r="D62" t="inlineStr">
         <is>
           <t>2021016402161952</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F62" t="n">
         <v>9.17</v>
       </c>
@@ -2089,13 +2557,21 @@
           <t>9041748</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>OMKAR MARUTI THORAT</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr">
         <is>
           <t>2021016402156943</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F63" t="n">
         <v>9.5</v>
       </c>
@@ -2115,13 +2591,21 @@
           <t>9041749</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>VAISHNAV VILAS THORWAT</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr">
         <is>
           <t>2021016402164111</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F64" t="n">
         <v>9.140000000000001</v>
       </c>
@@ -2141,13 +2625,21 @@
           <t>9041750</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>THOSAR MANAS MAHESH</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr">
         <is>
           <t>2021016402148425</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F65" t="n">
         <v>9.19</v>
       </c>
@@ -2167,13 +2659,21 @@
           <t>9041751</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>UTKARSH TIWARI</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr">
         <is>
           <t>2021016402158122</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F66" t="n">
         <v>9.140000000000001</v>
       </c>
@@ -2193,20 +2693,24 @@
           <t>9041752</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>RAHUL PREMSHANKAR YADAV</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr">
         <is>
           <t>2021016402160875</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>7.33</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H67" t="n">
         <v>218</v>
@@ -2221,13 +2725,21 @@
           <t>9041753</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr"/>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ADULKAR RUCHITA SHANKAR</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr">
         <is>
           <t>2021016402307694</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
       <c r="F68" t="n">
         <v>9.220000000000001</v>
       </c>
@@ -2281,7 +2793,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
@@ -2291,7 +2803,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>67</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>